<commit_message>
Automate recap pipeline: Bloomberg fetch, end-to-end runner, HTML output
- Add bloomberg_fetch.py: pull OPEN_INT_CHANGE + VOLUME via blpapi,
  replacing the manual Excel/BDP copy-paste step
- generate_recap_input_txt.py: source data from Bloomberg by default
  (--from-excel fallback); add "Trade Recap <prev business day>" header
- Add run_pipeline.py: run template -> tickers -> recap -> HTML end-to-end,
  while each step still runs standalone
- generate_trade_recap.py: accept "Volume =" delimiter in parse_volume_line
- Stop tracking __pycache__ bytecode (.gitignore)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/numbers.xlsx
+++ b/data/numbers.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wallachbeth-my.sharepoint.com/personal/ssaha_wallachbeth_com/Documents/Desktop/OI_Change_Tool/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{7FB34513-B051-4D77-8583-8DEB1B5BBDC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C1F9B9F-44B4-4C89-A5FD-EAB132C8149D}"/>
+  <xr:revisionPtr revIDLastSave="80" documentId="13_ncr:1_{7FB34513-B051-4D77-8583-8DEB1B5BBDC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A93388B-C580-419B-91E2-5FE58FF16E8E}"/>
   <bookViews>
-    <workbookView xWindow="39880" yWindow="3870" windowWidth="19430" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39990" yWindow="2420" windowWidth="18410" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="1">
   <si>
     <t>###</t>
   </si>
@@ -91,6 +91,101 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/volatileDependencies.xml><?xml version="1.0" encoding="utf-8"?>
+<volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <volType type="realTimeData">
+    <main first="bofaddin.rtdserver">
+      <tp>
+        <v>15288</v>
+        <stp/>
+        <stp>BDP|303756335481063149|22</stp>
+        <stp>WBD US 11/20/26 C28 Equity</stp>
+        <stp>VOLUME</stp>
+        <tr r="B7" s="1"/>
+      </tp>
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDP|16338704789380703350</stp>
+        <tr r="A8" s="1"/>
+      </tp>
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDP|10790127546866417927</stp>
+        <tr r="A1" s="1"/>
+      </tp>
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDP|13311422607760940446</stp>
+        <tr r="A5" s="1"/>
+      </tp>
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDP|12490645226751461408</stp>
+        <tr r="A9" s="1"/>
+      </tp>
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDP|14545488351304071131</stp>
+        <tr r="A7" s="1"/>
+      </tp>
+    </main>
+    <main first="bofaddin.rtdserver">
+      <tp>
+        <v>5486</v>
+        <stp/>
+        <stp>BDP|6070588607184154166|22</stp>
+        <stp>KVUE US 7/10/26 C20 Equity</stp>
+        <stp>VOLUME</stp>
+        <tr r="B1" s="1"/>
+      </tp>
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDP|2392720676065672016</stp>
+        <tr r="A3" s="1"/>
+      </tp>
+      <tp>
+        <v>418</v>
+        <stp/>
+        <stp>BDP|14969636648953227630|22</stp>
+        <stp>TECK US 7/17/26 C65 Equity</stp>
+        <stp>VOLUME</stp>
+        <tr r="B3" s="1"/>
+      </tp>
+      <tp>
+        <v>2003</v>
+        <stp/>
+        <stp>BDP|3576420985059501811|22</stp>
+        <stp>VAL US 8/21/26 C75 Equity</stp>
+        <stp>VOLUME</stp>
+        <tr r="B5" s="1"/>
+      </tp>
+      <tp>
+        <v>19647</v>
+        <stp/>
+        <stp>BDP|4058728448819540184|22</stp>
+        <stp>WBD US 8/21/26 C29 Equity</stp>
+        <stp>VOLUME</stp>
+        <tr r="B8" s="1"/>
+      </tp>
+      <tp>
+        <v>1106</v>
+        <stp/>
+        <stp>BDP|3392827669032419954|22</stp>
+        <stp>WBD US 8/21/26 P25 Equity</stp>
+        <stp>VOLUME</stp>
+        <tr r="B9" s="1"/>
+      </tp>
+    </main>
+  </volType>
+</volTypes>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -390,15 +485,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1">
-        <v>1336</v>
+        <f ca="1">IF($B1="","",_xll.BDP($B1,"open_int_change"))</f>
+        <v>-67</v>
       </c>
       <c r="B1">
-        <v>1600</v>
+        <f ca="1">IF($B1="","",_xll.BDP($B1,"VOLUME"))</f>
+        <v>5486</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -411,10 +508,12 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3">
-        <v>-13</v>
+        <f ca="1">IF($B3="","",_xll.BDP($B3,"open_int_change"))</f>
+        <v>163</v>
       </c>
       <c r="B3">
-        <v>2621</v>
+        <f ca="1">IF($B3="","",_xll.BDP($B3,"VOLUME"))</f>
+        <v>418</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -427,41 +526,57 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>20309</v>
+        <f ca="1">IF($B5="","",_xll.BDP($B5,"open_int_change"))</f>
+        <v>2000</v>
       </c>
       <c r="B5">
-        <v>20325</v>
+        <f ca="1">IF($B5="","",_xll.BDP($B5,"VOLUME"))</f>
+        <v>2003</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>-4099</v>
-      </c>
-      <c r="B6">
-        <v>12829</v>
+      <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7">
-        <v>5494</v>
+        <f ca="1">IF($B7="","",_xll.BDP($B7,"open_int_change"))</f>
+        <v>14964</v>
       </c>
       <c r="B7">
-        <v>8372</v>
+        <f ca="1">IF($B7="","",_xll.BDP($B7,"VOLUME"))</f>
+        <v>15288</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8">
-        <v>-2676</v>
+        <f ca="1">IF($B8="","",_xll.BDP($B8,"open_int_change"))</f>
+        <v>11521</v>
       </c>
       <c r="B8">
-        <v>4991</v>
+        <f ca="1">IF($B8="","",_xll.BDP($B8,"VOLUME"))</f>
+        <v>19647</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="A9">
+        <f ca="1">IF($B9="","",_xll.BDP($B9,"open_int_change"))</f>
+        <v>452</v>
+      </c>
+      <c r="B9">
+        <f ca="1">IF($B9="","",_xll.BDP($B9,"VOLUME"))</f>
+        <v>1106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>